<commit_message>
Filtro de guias +45
</commit_message>
<xml_diff>
--- a/Pruebas/Prueba1.xlsx
+++ b/Pruebas/Prueba1.xlsx
@@ -24,10 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
-  <si>
-    <t>numero_guia</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -430,26 +427,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
+      <c r="A1" s="3">
+        <v>46702592202</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
+      <c r="A3" s="3">
+        <v>46704880850</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>8</v>
+      <c r="A5" s="5">
+        <v>45704880850</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -458,11 +457,13 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
+      <c r="A7" s="4">
+        <v>46701695087</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -472,25 +473,30 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>45701695087</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -500,12 +506,12 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
@@ -518,9 +524,14 @@
         <v>45702592202</v>
       </c>
     </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>45701695087</v>
+      </c>
+    </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nuevos cambios version 1
</commit_message>
<xml_diff>
--- a/Pruebas/Prueba1.xlsx
+++ b/Pruebas/Prueba1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyecto\Pruebas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\El 498\Desktop\PYTHON\AMPMAuto\Pruebas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,26 +24,175 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>45704880850</t>
-  </si>
-  <si>
-    <t>45705084408</t>
-  </si>
-  <si>
-    <t>46701695087</t>
+    <t>47211807828</t>
+  </si>
+  <si>
+    <t>47219982378</t>
+  </si>
+  <si>
+    <t>47198179950</t>
+  </si>
+  <si>
+    <t>47207593653</t>
+  </si>
+  <si>
+    <t>47206817322</t>
+  </si>
+  <si>
+    <t>47211807852</t>
+  </si>
+  <si>
+    <t>47191718384</t>
+  </si>
+  <si>
+    <t>47212277835</t>
+  </si>
+  <si>
+    <t>47206563156</t>
+  </si>
+  <si>
+    <t>47212041827</t>
+  </si>
+  <si>
+    <t>47192686038</t>
+  </si>
+  <si>
+    <t>47197803721</t>
+  </si>
+  <si>
+    <t>47211292530</t>
+  </si>
+  <si>
+    <t>47218791855</t>
+  </si>
+  <si>
+    <t>47218656808</t>
+  </si>
+  <si>
+    <t>47215253452</t>
+  </si>
+  <si>
+    <t>47207577868</t>
+  </si>
+  <si>
+    <t>47216710911</t>
+  </si>
+  <si>
+    <t>47197080943</t>
+  </si>
+  <si>
+    <t>47218915981</t>
+  </si>
+  <si>
+    <t>47193537613</t>
+  </si>
+  <si>
+    <t>47216702068</t>
+  </si>
+  <si>
+    <t>47209335878</t>
+  </si>
+  <si>
+    <t>47168175889</t>
+  </si>
+  <si>
+    <t>47192440663</t>
+  </si>
+  <si>
+    <t>47212460228</t>
+  </si>
+  <si>
+    <t>47217422003</t>
+  </si>
+  <si>
+    <t>47216382695</t>
+  </si>
+  <si>
+    <t>47217814220</t>
+  </si>
+  <si>
+    <t>47216337176</t>
+  </si>
+  <si>
+    <t>47218876935</t>
+  </si>
+  <si>
+    <t>47218117104</t>
+  </si>
+  <si>
+    <t>47200607128</t>
+  </si>
+  <si>
+    <t>47218506657</t>
+  </si>
+  <si>
+    <t>47211319457</t>
+  </si>
+  <si>
+    <t>47215973832</t>
+  </si>
+  <si>
+    <t>47211311510</t>
+  </si>
+  <si>
+    <t>47199825010</t>
+  </si>
+  <si>
+    <t>47199866606</t>
+  </si>
+  <si>
+    <t>47178488340</t>
+  </si>
+  <si>
+    <t>47217700591</t>
+  </si>
+  <si>
+    <t>47215576099</t>
+  </si>
+  <si>
+    <t>47218470731</t>
+  </si>
+  <si>
+    <t>47215899559</t>
+  </si>
+  <si>
+    <t>47192673308</t>
+  </si>
+  <si>
+    <t>47218001782</t>
+  </si>
+  <si>
+    <t>47212565979</t>
+  </si>
+  <si>
+    <t>47199087295</t>
+  </si>
+  <si>
+    <t>47214247679</t>
+  </si>
+  <si>
+    <t>47212041793</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -71,11 +220,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -356,73 +506,266 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1">
-        <v>45709834061</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>46704880850</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13"/>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
       <c r="B13" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16"/>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>50</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>